<commit_message>
Add ACM and ScienceDirect export extension to query deliverables
</commit_message>
<xml_diff>
--- a/report/query_review_workbook.xlsx
+++ b/report/query_review_workbook.xlsx
@@ -2,13 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2a120cadc4a7498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R4f0e38b365c74947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included" sheetId="3" r:id="R480f3a01907a4fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="4" r:id="R501db9f2d4934ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downloads" sheetId="5" r:id="R35e7947e0149441e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Searches" sheetId="6" r:id="Rb5f4f9d0977e4ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Received" sheetId="7" r:id="Rfc86454e31cc4e7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R77b5262f6c7b4a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R56274c32e75f4bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included" sheetId="3" r:id="R137a082785d14329"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="4" r:id="Rfa978dd84c3d44ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downloads" sheetId="5" r:id="R8d11defedf0a4df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Searches" sheetId="6" r:id="R8af0b8958d6f4dd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Received" sheetId="7" r:id="R536c060475b641d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extension" sheetId="8" r:id="R2ddeddda07434f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NewQueue" sheetId="9" r:id="Re5321845250249c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,8 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -68,7 +71,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -84,6 +87,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -189,6 +195,40 @@
     <x:tableColumn id="4" name="Decision"/>
     <x:tableColumn id="5" name="QA"/>
     <x:tableColumn id="6" name="Source SHA256"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ExtensionTable" displayName="ExtensionTable" ref="A1:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Run"/>
+    <x:tableColumn id="2" name="Source"/>
+    <x:tableColumn id="3" name="Pakistan run time"/>
+    <x:tableColumn id="4" name="Displayed hits"/>
+    <x:tableColumn id="5" name="Claimed export"/>
+    <x:tableColumn id="6" name="Parsed entries"/>
+    <x:tableColumn id="7" name="Count difference: parsed - displayed"/>
+    <x:tableColumn id="8" name="Status / reconciliation"/>
+    <x:tableColumn id="9" name="Evidence"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="NewQueueTable" displayName="NewQueueTable" ref="A1:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Record"/>
+    <x:tableColumn id="2" name="Title"/>
+    <x:tableColumn id="3" name="Year"/>
+    <x:tableColumn id="4" name="DOI"/>
+    <x:tableColumn id="5" name="Decision"/>
+    <x:tableColumn id="6" name="Date check"/>
+    <x:tableColumn id="7" name="Full text"/>
+    <x:tableColumn id="8" name="Study status"/>
+    <x:tableColumn id="9" name="Source file"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -25893,7 +25933,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5a430e8f2f44b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc15c9c329b4d4a83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26420,7 +26460,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11fb79c6e4674bd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c72be1699664967"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27458,7 +27498,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cde3691092e4ecf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92cb66593eea4a88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29418,7 +29458,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbe0c826b3c04c6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf6eff9b246a402f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29674,7 +29714,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcb9ec48088b4ec9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87dcec69ebe944b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29834,7 +29874,792 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5806c7b7af304478"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b673200c874e61"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="85" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="75" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Run</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Pakistan run time</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>Displayed hits</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>Claimed export</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Parsed entries</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>Count difference: parsed - displayed</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Status / reconciliation</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="75" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>ACM-MASTER</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>ACM Digital Library (The ACM Full-Text Collection)</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>14 October 2026, 10:30 PM</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="n">
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="n">
+        <x:v>1603</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="n">
+        <x:v>1829</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="n">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>1600 displayed; 1603 claimed exported; 1829 parsed in two master files; page ranges/extra records unverified</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="str">
+        <x:v>search_runs_received.csv / export_intake.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="75" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>SD-TEMPORAL</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>ScienceDirect</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>14 October 2026, 11:45 PM</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="n">
+        <x:v>1053</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="n">
+        <x:v>1053</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="n">
+        <x:v>1053</x:v>
+      </x:c>
+      <x:c r="G3" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="str">
+        <x:v>URL includes openaccess facet absent from written filter description; confirm applied facet</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="str">
+        <x:v>search_runs_received.csv / export_intake.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="75" customHeight="1">
+      <x:c r="A4" s="2" t="str">
+        <x:v>SD-MPS</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>ScienceDirect</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>14 October 2026, 11:52 PM</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="n">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="E4" s="7" t="n">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="F4" s="7" t="n">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="G4" s="7" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="H4" s="2" t="str">
+        <x:v>517 displayed; 563 parsed/exported; investigate count or selection mismatch</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="str">
+        <x:v>search_runs_received.csv / export_intake.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="75" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>SD-MIG</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>ScienceDirect</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>14 October 2026, 11:55 PM</x:v>
+      </x:c>
+      <x:c r="D5" s="7" t="n">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="n">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="F5" s="7" t="n">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="G5" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="2" t="str">
+        <x:v>Values agree; protocol cutoff still requires screening</x:v>
+      </x:c>
+      <x:c r="I5" s="2" t="str">
+        <x:v>search_runs_received.csv / export_intake.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="75" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>SD-API</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>ScienceDirect</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>14 October 2026, 11:56 PM</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="G6" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="2" t="str">
+        <x:v>Values agree; protocol cutoff still requires screening</x:v>
+      </x:c>
+      <x:c r="I6" s="2" t="str">
+        <x:v>search_runs_received.csv / export_intake.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="75" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>TOTAL</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>Five supplied runs</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>2026-10-14</x:v>
+      </x:c>
+      <x:c r="D7" s="7" t="n">
+        <x:v>3452</x:v>
+      </x:c>
+      <x:c r="E7" s="7" t="n">
+        <x:v>3501</x:v>
+      </x:c>
+      <x:c r="F7" s="7" t="n">
+        <x:v>3727</x:v>
+      </x:c>
+      <x:c r="G7" s="7" t="n">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="H7" s="2" t="str">
+        <x:v>Occurrence totals; not deduplicated or a revised PRISMA flow</x:v>
+      </x:c>
+      <x:c r="I7" s="2" t="str">
+        <x:v>new_export_occurrences.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="75" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>REVIEW</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>23 files; 3,727 new occurrences</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D8" s="2"/>
+      <x:c r="E8" s="2"/>
+      <x:c r="F8" s="2"/>
+      <x:c r="G8" s="2"/>
+      <x:c r="H8" s="2" t="str">
+        <x:v>6 title/abstract exclusions; 12 queued for full text; 3,709 without decision; 21 previously accepted studies unchanged</x:v>
+      </x:c>
+      <x:c r="I8" s="2" t="str">
+        <x:v>priority_title_abstract_decisions.csv / priority_fulltext_queue.csv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a2c2546b8554893"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="82" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="80" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="80" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Record</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Title</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>DOI</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Date check</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>Full text</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Study status</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Source file</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="80" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>GA-N00001</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>MIGER: Integrating Multi-Instance GPU and Multi-Process Service for Deep Learning Clusters</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>10.1145/3673038.3673089</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="80" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>GA-N00005</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>Towards Optimal Preemptive GPU Time-Sharing for Edge Model Serving</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>10.1145/3631311.3632401</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="80" customHeight="1">
+      <x:c r="A4" s="2" t="str">
+        <x:v>GA-N00015</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>FaST-GShare: Enabling Efficient Spatio-Temporal GPU Sharing in Serverless Computing for Deep Learning Inference</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>10.1145/3605573.3605638</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H4" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="80" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>GA-N00029</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>Pantheon: Preemptible Multi-DNN Inference on Mobile Edge GPUs</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="str">
+        <x:v>10.1145/3643832.3661878</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H5" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I5" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="80" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>GA-N00040</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>SPLIT: QoS-Aware DNN Inference on Shared GPU via Evenly-Sized Model Splitting</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>10.1145/3605573.3605627</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F6" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G6" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H6" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I6" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="80" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>GA-N00043</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>Optimizing GPU Sharing for Container-Based DNN Serving with Multi-Instance GPUs</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="str">
+        <x:v>10.1145/3688351.3689156</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G7" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H7" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I7" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="80" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>GA-N00831</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>MIGServe: Layout-Aware Multi-Instance GPU Management for Efficient LLM Serving</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="str">
+        <x:v>10.1145/3832810.3832898</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="str">
+        <x:v>verify exact publication date against 11 October 2026 cutoff</x:v>
+      </x:c>
+      <x:c r="G8" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H8" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I8" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="80" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>GA-N00839</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>MMK: A Hybrid Scheduling Framework for Fine-Grained GPU Sharing for Deep Learning Applications</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>10.1145/3820163</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="str">
+        <x:v>verify exact publication date against 11 October 2026 cutoff</x:v>
+      </x:c>
+      <x:c r="G9" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H9" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I9" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="80" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>GA-N00844</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>BOER: Enhancing Resource Utilization for Deep Learning Inference with Hybrid Spatial GPU Sharing</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>10.1145/3712285.3759857</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H10" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="80" customHeight="1">
+      <x:c r="A11" s="2" t="str">
+        <x:v>GA-N00872</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>Adaptive GPU Sharing for Real-time LLM Serving with Best-effort Workloads</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>10.1145/3816891.3834895</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="str">
+        <x:v>verify exact publication date against 11 October 2026 cutoff</x:v>
+      </x:c>
+      <x:c r="G11" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H11" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I11" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="80" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>GA-N00904</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>SGDRC: Software-Defined Dynamic Resource Control for Concurrent DNN Inference on NVIDIA GPUs</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>10.1145/3710848.3710863</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="str">
+        <x:v>year within period</x:v>
+      </x:c>
+      <x:c r="G12" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H12" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I12" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="80" customHeight="1">
+      <x:c r="A13" s="2" t="str">
+        <x:v>GA-N00946</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>Beyond Utilization: Energy-Conscious GPU Sharing for Inference Serving</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>10.1145/3830418.3843913</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>retrieve_for_eligibility</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>verify exact publication date against 11 October 2026 cutoff</x:v>
+      </x:c>
+      <x:c r="G13" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H13" s="2" t="str">
+        <x:v>candidate, not included</x:v>
+      </x:c>
+      <x:c r="I13" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="80" customHeight="1">
+      <x:c r="A14" s="2" t="str">
+        <x:v>GA-N00013</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>Deep Learning Workload Scheduling in GPU Datacenters: A Survey</x:v>
+      </x:c>
+      <x:c r="C14" s="2"/>
+      <x:c r="D14" s="2" t="str"/>
+      <x:c r="E14" s="2" t="str">
+        <x:v>exclude at title_abstract</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="str"/>
+      <x:c r="G14" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H14" s="2" t="str">
+        <x:v>not included; E6: Survey; not an original primary evaluation.</x:v>
+      </x:c>
+      <x:c r="I14" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="80" customHeight="1">
+      <x:c r="A15" s="2" t="str">
+        <x:v>GA-N00030</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>Online evolutionary batch size orchestration for scheduling deep learning workloads in GPU clusters</x:v>
+      </x:c>
+      <x:c r="C15" s="2"/>
+      <x:c r="D15" s="2" t="str"/>
+      <x:c r="E15" s="2" t="str">
+        <x:v>exclude at title_abstract</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="str"/>
+      <x:c r="G15" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H15" s="2" t="str">
+        <x:v>not included; E4: Abstract addresses deep-learning training cost and cluster scheduling, without inference-serving evidence.</x:v>
+      </x:c>
+      <x:c r="I15" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="80" customHeight="1">
+      <x:c r="A16" s="2" t="str">
+        <x:v>GA-N00069</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>Characterizing Training Performance and Energy for Foundation Models and Image Classifiers on Multi-Instance GPUs</x:v>
+      </x:c>
+      <x:c r="C16" s="2"/>
+      <x:c r="D16" s="2" t="str"/>
+      <x:c r="E16" s="2" t="str">
+        <x:v>exclude at title_abstract</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="str"/>
+      <x:c r="G16" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H16" s="2" t="str">
+        <x:v>not included; E4: Title/abstract characterize training performance and energy on MIG, without inference-serving evidence.</x:v>
+      </x:c>
+      <x:c r="I16" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="80" customHeight="1">
+      <x:c r="A17" s="2" t="str">
+        <x:v>GA-N00081</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>Kale: Elastic GPU Scheduling for Online DL Model Training</x:v>
+      </x:c>
+      <x:c r="C17" s="2"/>
+      <x:c r="D17" s="2" t="str"/>
+      <x:c r="E17" s="2" t="str">
+        <x:v>exclude at title_abstract</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str"/>
+      <x:c r="G17" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H17" s="2" t="str">
+        <x:v>not included; E4: Title/abstract concern online and offline model training scheduling.</x:v>
+      </x:c>
+      <x:c r="I17" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="80" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>GA-N00092</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>RAP: Resource-aware Automated GPU Sharing for Multi-GPU Recommendation Model Training and Input Preprocessing</x:v>
+      </x:c>
+      <x:c r="C18" s="2"/>
+      <x:c r="D18" s="2" t="str"/>
+      <x:c r="E18" s="2" t="str">
+        <x:v>exclude at title_abstract</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str"/>
+      <x:c r="G18" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H18" s="2" t="str">
+        <x:v>not included; E4: Title/abstract concern recommendation-model retraining and input preprocessing.</x:v>
+      </x:c>
+      <x:c r="I18" s="2" t="str">
+        <x:v>ACM_MASTER_01.bib</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="80" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>GA-N00874</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>Performance Prediction of Concurrent DNN Training Tasks in GPU Spatial Sharing Environments</x:v>
+      </x:c>
+      <x:c r="C19" s="2"/>
+      <x:c r="D19" s="2" t="str"/>
+      <x:c r="E19" s="2" t="str">
+        <x:v>exclude at title_abstract</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str"/>
+      <x:c r="G19" s="2" t="str">
+        <x:v>not assessed</x:v>
+      </x:c>
+      <x:c r="H19" s="2" t="str">
+        <x:v>not included; E4: Title/abstract concern concurrent DNN training task prediction.</x:v>
+      </x:c>
+      <x:c r="I19" s="2" t="str">
+        <x:v>ACM_MASTER_02.bib</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3e2c78149504574"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>